<commit_message>
Bulk update 2026-06-11: new repos, consumer AI, tech news, papers
- Add Odysseus (PewDiePie), bug trivia, programmer meme
- Add consumer brand AI tools research (瑞幸/喜茶/星巴克/肯德基/海底捞等)
- Add 2026 AI/semiconductor/stock news summary (Jan-Jun)
- Add top conference papers (CVPR/ICLR/ICML/ACL/MLSys)
- Add categorized folders and archive structure
- Rewrite README with personality

🤖 Generated with [Qoder][https://qoder.com]
</commit_message>
<xml_diff>
--- a/favorites.xlsx
+++ b/favorites.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="效率小技巧" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="热门开源仓库" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技术冷知识" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="程序员梗" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58,11 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +510,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>find 的 Rust 替代品，秒级模糊查找文件</t>
+          <t>find的Rust替代品，秒级模糊查找文件</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -517,7 +520,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>fd /config.*ts/</t>
+          <t>fd "config.*ts"</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -554,7 +557,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>grep 的极速替代品，代码搜索利器</t>
+          <t>grep的极速替代品，代码搜索利器</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -564,7 +567,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>rg /TODO/ --type js</t>
+          <t>rg "TODO" --type js</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -594,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -667,7 +670,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>从AI玩具进化成实用开发工具，能帮你在重构时少踩坑</t>
+          <t>从AI玩具进化成实用开发工具</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -766,6 +769,44 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>repo-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Odysseus</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>自托管AI工作台，统一管理所有AI订阅和本地大模型</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>YouTube顶流PewDiePie随手搓出来的工具，4天狂揽5万多GitHub Star</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ai,self-hosted,llm,pewdiepie</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>viral</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>2026-06-11</t>
         </is>
@@ -782,20 +823,159 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>标题</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>标签</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>添加日期</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>trivia-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>世界上第一个bug真的是只虫子</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1947年9月，Grace Hopper在Harvard Mark II计算机的继电器触点里发现了一只烤焦的飞蛾，她把飞蛾尸体贴在工作日志上，写着：First actual case of bug being found.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>history,bug,grace-hopper</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>标签</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>添加日期</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>meme-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>My code doesn't work, I don't know why. My code works, I don't know why.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>programmer,debugging</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>新增内容</t>
         </is>
@@ -809,7 +989,55 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>初始创建：fd、ripgrep技巧 + OpenDevin-Next、LocalLLM-Runtime、Hono-X仓库</t>
+          <t>初始创建</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>追加：Odysseus + 第一个bug冷知识 + 程序员梗</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>新增：消费品牌AI工具调研</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>新增：2026年AI/半导体/芯片/股市新闻汇总</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>新增：2026年顶会论文汇总（CVPR/ICLR/ICML/ACL/MLSys）</t>
         </is>
       </c>
     </row>

</xml_diff>